<commit_message>
Add SQL script for customer, orders, and employees tables with sample data
</commit_message>
<xml_diff>
--- a/Excel/Final_Exam/matches.xlsx
+++ b/Excel/Final_Exam/matches.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Priyansh\OneDrive\Desktop\RW_Exam\Excel\Final_Exam\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{DAC254E6-401C-4967-A448-EC27EB77587A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:9_{46B15981-FE37-433F-BB61-CAF8BD40B499}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{970DA121-ED4C-4F36-8E52-DF73BA9A9F69}"/>
+    <workbookView minimized="1" xWindow="5760" yWindow="3360" windowWidth="17280" windowHeight="8880" xr2:uid="{970DA121-ED4C-4F36-8E52-DF73BA9A9F69}"/>
   </bookViews>
   <sheets>
     <sheet name="matches" sheetId="1" r:id="rId1"/>
@@ -2408,6 +2408,18 @@
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{58D2FFA6-834D-40C3-90D9-1CDE1B628961}">
   <dimension ref="A1:T1096"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="4" max="4" width="12.21875" customWidth="1"/>
+    <col min="6" max="6" width="17" customWidth="1"/>
+    <col min="7" max="7" width="36.6640625" customWidth="1"/>
+    <col min="8" max="8" width="25.5546875" customWidth="1"/>
+    <col min="9" max="9" width="24.88671875" customWidth="1"/>
+    <col min="10" max="10" width="26.109375" customWidth="1"/>
+    <col min="11" max="11" width="15.33203125" customWidth="1"/>
+    <col min="12" max="12" width="18.77734375" customWidth="1"/>
+    <col min="14" max="14" width="13.44140625" customWidth="1"/>
+    <col min="15" max="15" width="15.77734375" customWidth="1"/>
+  </cols>
   <sheetData>
     <row r="1" spans="1:20" x14ac:dyDescent="0.3">
       <c r="A1" t="s">

</xml_diff>